<commit_message>
updated for cell references
</commit_message>
<xml_diff>
--- a/excel/excel-101/MonthlyBudget.xlsx
+++ b/excel/excel-101/MonthlyBudget.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rajkhare/Raj/Udemy/ms-office/excel/excel-101/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5258C671-E7D6-0D41-91F0-B3A6F0FA70D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{351012BE-6DEA-0F43-BF21-B7FD0F83FA40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16780" xr2:uid="{61CE2942-B3C2-844E-8245-A989A6B80F58}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>Monthly Budget</t>
   </si>
@@ -56,15 +56,6 @@
   </si>
   <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t>Jan</t>
-  </si>
-  <si>
-    <t>Feb</t>
-  </si>
-  <si>
-    <t>Mar</t>
   </si>
   <si>
     <t>Petrol</t>
@@ -83,6 +74,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="mmm\-yyyy"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -112,8 +106,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -443,14 +438,14 @@
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
+      <c r="B3" s="1">
+        <v>45658</v>
+      </c>
+      <c r="C3" s="1">
+        <v>45689</v>
+      </c>
+      <c r="D3" s="1">
+        <v>45717</v>
       </c>
       <c r="E3" t="s">
         <v>6</v>
@@ -514,7 +509,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>1500</v>
@@ -528,7 +523,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B9">
         <v>5000</v>
@@ -542,7 +537,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B10">
         <v>6000</v>
@@ -556,7 +551,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B11">
         <v>600</v>

</xml_diff>

<commit_message>
Relative vs Absolute cell references
</commit_message>
<xml_diff>
--- a/excel/excel-101/MonthlyBudget.xlsx
+++ b/excel/excel-101/MonthlyBudget.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rajkhare/Raj/Udemy/ms-office/excel/excel-101/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{351012BE-6DEA-0F43-BF21-B7FD0F83FA40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3CC6595-2649-1542-A7E7-33517E705AD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16780" xr2:uid="{61CE2942-B3C2-844E-8245-A989A6B80F58}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>Monthly Budget</t>
   </si>
@@ -68,6 +68,9 @@
   </si>
   <si>
     <t>Entertainment</t>
+  </si>
+  <si>
+    <t>Percent</t>
   </si>
 </sst>
 </file>
@@ -75,7 +78,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="mmm\-yyyy"/>
+    <numFmt numFmtId="164" formatCode="mmm\-yyyy"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -108,7 +111,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -423,18 +426,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53CFA12A-055A-DD46-B8BC-7BBA25CD28AE}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -450,8 +453,11 @@
       <c r="E3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -464,8 +470,16 @@
       <c r="D4">
         <v>19000</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E4">
+        <f>B4+C4+D4</f>
+        <v>57000</v>
+      </c>
+      <c r="F4">
+        <f>(E4/$E$12)*100</f>
+        <v>34.915773353751916</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -478,8 +492,16 @@
       <c r="D5">
         <v>600</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E5">
+        <f>B5+C5+D5</f>
+        <v>1800</v>
+      </c>
+      <c r="F5">
+        <f>(E5/$E$12)*100</f>
+        <v>1.1026033690658499</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -492,8 +514,16 @@
       <c r="D6">
         <v>8000</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E6">
+        <f>B6+C6+D6</f>
+        <v>23000</v>
+      </c>
+      <c r="F6">
+        <f>(E6/$E$12)*100</f>
+        <v>14.088820826952528</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -506,8 +536,16 @@
       <c r="D7">
         <v>14000</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E7">
+        <f>B7+C7+D7</f>
+        <v>43000</v>
+      </c>
+      <c r="F7">
+        <f>(E7/$E$12)*100</f>
+        <v>26.339969372128635</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -520,8 +558,16 @@
       <c r="D8">
         <v>1200</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E8">
+        <f>B8+C8+D8</f>
+        <v>3900</v>
+      </c>
+      <c r="F8">
+        <f t="shared" ref="F5:F12" si="0">(E8/$E$12)*100</f>
+        <v>2.3889739663093414</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -534,8 +580,16 @@
       <c r="D9">
         <v>5000</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E9">
+        <f>B9+C9+D9</f>
+        <v>15000</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>9.1883614088820824</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -548,13 +602,21 @@
       <c r="D10">
         <v>6000</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E10">
+        <f>B10+C10+D10</f>
+        <v>18000</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>11.026033690658499</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11">
-        <v>600</v>
+        <v>450</v>
       </c>
       <c r="C11">
         <v>500</v>
@@ -562,10 +624,38 @@
       <c r="D11">
         <v>600</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E11">
+        <f>B11+C11+D11</f>
+        <v>1550</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>0.94946401225114863</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>6</v>
+      </c>
+      <c r="B12">
+        <f>B4+B5+B6+B7+B8+B9+B10+B11</f>
+        <v>54550</v>
+      </c>
+      <c r="C12">
+        <f>C4+C5+C6+C7+C8+C9+C10+C11</f>
+        <v>54300</v>
+      </c>
+      <c r="D12">
+        <f>D4+D5+D6+D7+D8+D9+D10+D11</f>
+        <v>54400</v>
+      </c>
+      <c r="E12">
+        <f>B12+C12+D12</f>
+        <v>163250</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modifying an Excel sheet
</commit_message>
<xml_diff>
--- a/excel/excel-101/MonthlyBudget.xlsx
+++ b/excel/excel-101/MonthlyBudget.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rajkhare/Raj/Udemy/ms-office/excel/excel-101/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACA51AC9-6CAA-D949-8219-7ACBA01FEE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD93A9C3-9192-CA49-B9F2-D0C9D83620FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16780" xr2:uid="{61CE2942-B3C2-844E-8245-A989A6B80F58}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="16">
   <si>
     <t>Monthly Budget</t>
   </si>
@@ -80,6 +81,9 @@
   </si>
   <si>
     <t>AVERAGE</t>
+  </si>
+  <si>
+    <t>COUNT</t>
   </si>
 </sst>
 </file>
@@ -435,11 +439,338 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53CFA12A-055A-DD46-B8BC-7BBA25CD28AE}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="B2:G17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1">
+        <v>45658</v>
+      </c>
+      <c r="D4" s="1">
+        <v>45689</v>
+      </c>
+      <c r="E4" s="1">
+        <v>45717</v>
+      </c>
+      <c r="F4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>19000</v>
+      </c>
+      <c r="D5">
+        <v>19000</v>
+      </c>
+      <c r="E5">
+        <v>19000</v>
+      </c>
+      <c r="F5">
+        <f>SUM(C5:E5)</f>
+        <v>57000</v>
+      </c>
+      <c r="G5">
+        <f>(F5/$F$13)*100</f>
+        <v>34.915773353751916</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>600</v>
+      </c>
+      <c r="D6">
+        <v>600</v>
+      </c>
+      <c r="E6">
+        <v>600</v>
+      </c>
+      <c r="F6">
+        <f>SUM(C6:E6)</f>
+        <v>1800</v>
+      </c>
+      <c r="G6">
+        <f>(F6/$F$13)*100</f>
+        <v>1.1026033690658499</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>8000</v>
+      </c>
+      <c r="D7">
+        <v>7000</v>
+      </c>
+      <c r="E7">
+        <v>8000</v>
+      </c>
+      <c r="F7">
+        <f>SUM(C7:E7)</f>
+        <v>23000</v>
+      </c>
+      <c r="G7">
+        <f>(F7/$F$13)*100</f>
+        <v>14.088820826952528</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8">
+        <v>14000</v>
+      </c>
+      <c r="D8">
+        <v>15000</v>
+      </c>
+      <c r="E8">
+        <v>14000</v>
+      </c>
+      <c r="F8">
+        <f>SUM(C8:E8)</f>
+        <v>43000</v>
+      </c>
+      <c r="G8">
+        <f>(F8/$F$13)*100</f>
+        <v>26.339969372128635</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <v>1500</v>
+      </c>
+      <c r="D9">
+        <v>1200</v>
+      </c>
+      <c r="E9">
+        <v>1200</v>
+      </c>
+      <c r="F9">
+        <f>SUM(C9:E9)</f>
+        <v>3900</v>
+      </c>
+      <c r="G9">
+        <f>(F9/$F$13)*100</f>
+        <v>2.3889739663093414</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10">
+        <v>5000</v>
+      </c>
+      <c r="D10">
+        <v>5000</v>
+      </c>
+      <c r="E10">
+        <v>5000</v>
+      </c>
+      <c r="F10">
+        <f>SUM(C10:E10)</f>
+        <v>15000</v>
+      </c>
+      <c r="G10">
+        <f>(F10/$F$13)*100</f>
+        <v>9.1883614088820824</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11">
+        <v>6000</v>
+      </c>
+      <c r="D11">
+        <v>6000</v>
+      </c>
+      <c r="E11">
+        <v>6000</v>
+      </c>
+      <c r="F11">
+        <f>SUM(C11:E11)</f>
+        <v>18000</v>
+      </c>
+      <c r="G11">
+        <f>(F11/$F$13)*100</f>
+        <v>11.026033690658499</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12">
+        <v>450</v>
+      </c>
+      <c r="D12">
+        <v>500</v>
+      </c>
+      <c r="E12">
+        <v>600</v>
+      </c>
+      <c r="F12">
+        <f>SUM(C12:E12)</f>
+        <v>1550</v>
+      </c>
+      <c r="G12">
+        <f>(F12/$F$13)*100</f>
+        <v>0.94946401225114863</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13">
+        <f>SUM(C5:C12)</f>
+        <v>54550</v>
+      </c>
+      <c r="D13">
+        <f t="shared" ref="D13:F13" si="0">SUM(D5:D12)</f>
+        <v>54300</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>54400</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>163250</v>
+      </c>
+      <c r="G13">
+        <f>(F13/$F$13)*100</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14">
+        <f>MIN(C5:C12)</f>
+        <v>450</v>
+      </c>
+      <c r="D14">
+        <f>MIN(D5:D12)</f>
+        <v>500</v>
+      </c>
+      <c r="E14">
+        <f>MIN(E5:E12)</f>
+        <v>600</v>
+      </c>
+      <c r="F14">
+        <f>MIN(F5:F12)</f>
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15">
+        <f>MAX(C5:C12)</f>
+        <v>19000</v>
+      </c>
+      <c r="D15">
+        <f>MAX(D5:D12)</f>
+        <v>19000</v>
+      </c>
+      <c r="E15">
+        <f>MAX(E5:E12)</f>
+        <v>19000</v>
+      </c>
+      <c r="F15">
+        <f>MAX(F5:F12)</f>
+        <v>57000</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16">
+        <f>AVERAGE(C5:C12)</f>
+        <v>6818.75</v>
+      </c>
+      <c r="D16">
+        <f>AVERAGE(D5:D12)</f>
+        <v>6787.5</v>
+      </c>
+      <c r="E16">
+        <f>AVERAGE(E5:E12)</f>
+        <v>6800</v>
+      </c>
+      <c r="F16">
+        <f>AVERAGE(F5:F12)</f>
+        <v>20406.25</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17">
+        <f>COUNT(C5:C12)</f>
+        <v>8</v>
+      </c>
+      <c r="D17">
+        <f>COUNT(D5:D12)</f>
+        <v>8</v>
+      </c>
+      <c r="E17">
+        <f>COUNT(E5:E12)</f>
+        <v>8</v>
+      </c>
+      <c r="F17">
+        <f>COUNT(F5:F12)</f>
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="C13:E13 C14:E17" formulaRange="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C881B40-3868-B64D-BC40-E4666107B0E3}">
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -480,12 +811,12 @@
         <v>19000</v>
       </c>
       <c r="E4">
-        <f t="shared" ref="E4:E11" si="0">SUM(B4:D4)</f>
+        <f>SUM(B4:D4)</f>
         <v>57000</v>
       </c>
-      <c r="F4">
-        <f>(E4/$E$12)*100</f>
-        <v>34.915773353751916</v>
+      <c r="F4" t="e">
+        <f>(E4/$H$14)*100</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -502,12 +833,12 @@
         <v>600</v>
       </c>
       <c r="E5">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E5:E11" si="0">SUM(B5:D5)</f>
         <v>1800</v>
       </c>
-      <c r="F5">
-        <f>(E5/$E$12)*100</f>
-        <v>1.1026033690658499</v>
+      <c r="F5" t="e">
+        <f>(E5/$H$14)*100</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -527,9 +858,9 @@
         <f t="shared" si="0"/>
         <v>23000</v>
       </c>
-      <c r="F6">
-        <f>(E6/$E$12)*100</f>
-        <v>14.088820826952528</v>
+      <c r="F6" t="e">
+        <f>(E6/$H$14)*100</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -549,9 +880,9 @@
         <f t="shared" si="0"/>
         <v>43000</v>
       </c>
-      <c r="F7">
-        <f>(E7/$E$12)*100</f>
-        <v>26.339969372128635</v>
+      <c r="F7" t="e">
+        <f>(E7/$H$14)*100</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -571,9 +902,9 @@
         <f t="shared" si="0"/>
         <v>3900</v>
       </c>
-      <c r="F8">
-        <f t="shared" ref="F8:F12" si="1">(E8/$E$12)*100</f>
-        <v>2.3889739663093414</v>
+      <c r="F8" t="e">
+        <f>(E8/$H$14)*100</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -593,9 +924,9 @@
         <f t="shared" si="0"/>
         <v>15000</v>
       </c>
-      <c r="F9">
-        <f t="shared" si="1"/>
-        <v>9.1883614088820824</v>
+      <c r="F9" t="e">
+        <f>(E9/$H$14)*100</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -615,9 +946,9 @@
         <f t="shared" si="0"/>
         <v>18000</v>
       </c>
-      <c r="F10">
-        <f t="shared" si="1"/>
-        <v>11.026033690658499</v>
+      <c r="F10" t="e">
+        <f>(E10/$H$14)*100</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -637,9 +968,9 @@
         <f t="shared" si="0"/>
         <v>1550</v>
       </c>
-      <c r="F11">
-        <f t="shared" si="1"/>
-        <v>0.94946401225114863</v>
+      <c r="F11" t="e">
+        <f>(E11/$H$14)*100</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -651,20 +982,20 @@
         <v>54550</v>
       </c>
       <c r="C12">
-        <f>SUM(C4:C11)</f>
+        <f t="shared" ref="C12:E12" si="1">SUM(C4:C11)</f>
         <v>54300</v>
       </c>
       <c r="D12">
-        <f>SUM(D4:D11)</f>
+        <f t="shared" si="1"/>
         <v>54400</v>
       </c>
       <c r="E12">
-        <f>SUM(E4:E11)</f>
+        <f t="shared" si="1"/>
         <v>163250</v>
       </c>
-      <c r="F12">
-        <f t="shared" si="1"/>
-        <v>100</v>
+      <c r="F12" t="e">
+        <f>(E12/$H$14)*100</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -687,10 +1018,6 @@
         <f>MIN(E4:E11)</f>
         <v>1550</v>
       </c>
-      <c r="F14">
-        <f>MIN(F4:F11)</f>
-        <v>0.94946401225114863</v>
-      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -712,10 +1039,6 @@
         <f>MAX(E4:E11)</f>
         <v>57000</v>
       </c>
-      <c r="F15">
-        <f>MAX(F4:F11)</f>
-        <v>34.915773353751916</v>
-      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -737,15 +1060,29 @@
         <f>AVERAGE(E4:E11)</f>
         <v>20406.25</v>
       </c>
-      <c r="F16">
-        <f>AVERAGE(F4:F11)</f>
-        <v>12.5</v>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <f>COUNT(B4:B11)</f>
+        <v>8</v>
+      </c>
+      <c r="C17">
+        <f>COUNT(C4:C11)</f>
+        <v>8</v>
+      </c>
+      <c r="D17">
+        <f>COUNT(D4:D11)</f>
+        <v>8</v>
+      </c>
+      <c r="E17">
+        <f>COUNT(E4:E11)</f>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="B12:D12 B14:B16 C14:D16" formulaRange="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added for excel formatting
</commit_message>
<xml_diff>
--- a/excel/excel-101/MonthlyBudget.xlsx
+++ b/excel/excel-101/MonthlyBudget.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rajkhare/Raj/Udemy/ms-office/excel/excel-101/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD93A9C3-9192-CA49-B9F2-D0C9D83620FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{493BA6E0-DE8E-AD49-8FEE-B3E06BA69D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16780" xr2:uid="{61CE2942-B3C2-844E-8245-A989A6B80F58}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16720" xr2:uid="{61CE2942-B3C2-844E-8245-A989A6B80F58}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Monthly Budget" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>Monthly Budget</t>
   </si>
@@ -90,10 +89,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="4">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="mmm\-yyyy"/>
+    <numFmt numFmtId="165" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -101,16 +103,55 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="0"/>
+      <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -118,16 +159,53 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyNumberFormat="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="3"/>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="2" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="4">
+    <cellStyle name="AwesomeStyle" xfId="3" xr:uid="{0FC19754-6B15-7D41-8A87-4B406E4C2DC9}"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -439,650 +517,342 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53CFA12A-055A-DD46-B8BC-7BBA25CD28AE}">
-  <dimension ref="B2:G17"/>
+  <dimension ref="B1:G18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B2" t="s">
+    <row r="1" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="F1" s="8"/>
+    </row>
+    <row r="2" spans="2:7" ht="37" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+    </row>
+    <row r="3" spans="2:7" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="4" spans="2:7" ht="26" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="6">
         <v>45658</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="6">
         <v>45689</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="6">
         <v>45717</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:7" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>2</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="1">
         <v>19000</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="1">
         <v>19000</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="1">
         <v>19000</v>
       </c>
-      <c r="F5">
-        <f>SUM(C5:E5)</f>
+      <c r="F5" s="1">
+        <f t="shared" ref="F5:F12" si="0">SUM(C5:E5)</f>
         <v>57000</v>
       </c>
-      <c r="G5">
-        <f>(F5/$F$13)*100</f>
-        <v>34.915773353751916</v>
+      <c r="G5" s="3">
+        <f>(F5/$F$13)</f>
+        <v>0.34915773353751917</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>3</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="2">
         <v>600</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <v>600</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="2">
         <v>600</v>
       </c>
-      <c r="F6">
-        <f>SUM(C6:E6)</f>
+      <c r="F6" s="2">
+        <f t="shared" si="0"/>
         <v>1800</v>
       </c>
-      <c r="G6">
-        <f>(F6/$F$13)*100</f>
-        <v>1.1026033690658499</v>
+      <c r="G6" s="3">
+        <f t="shared" ref="G6:G12" si="1">(F6/$F$13)</f>
+        <v>1.1026033690658498E-2</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>4</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="2">
         <v>8000</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="2">
         <v>7000</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="2">
         <v>8000</v>
       </c>
-      <c r="F7">
-        <f>SUM(C7:E7)</f>
+      <c r="F7" s="2">
+        <f t="shared" si="0"/>
         <v>23000</v>
       </c>
-      <c r="G7">
-        <f>(F7/$F$13)*100</f>
-        <v>14.088820826952528</v>
+      <c r="G7" s="3">
+        <f t="shared" si="1"/>
+        <v>0.14088820826952528</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>5</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="2">
         <v>14000</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="2">
         <v>15000</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="2">
         <v>14000</v>
       </c>
-      <c r="F8">
-        <f>SUM(C8:E8)</f>
+      <c r="F8" s="2">
+        <f t="shared" si="0"/>
         <v>43000</v>
       </c>
-      <c r="G8">
-        <f>(F8/$F$13)*100</f>
-        <v>26.339969372128635</v>
+      <c r="G8" s="3">
+        <f t="shared" si="1"/>
+        <v>0.26339969372128635</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>7</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="2">
         <v>1500</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="2">
         <v>1200</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="2">
         <v>1200</v>
       </c>
-      <c r="F9">
-        <f>SUM(C9:E9)</f>
+      <c r="F9" s="2">
+        <f t="shared" si="0"/>
         <v>3900</v>
       </c>
-      <c r="G9">
-        <f>(F9/$F$13)*100</f>
-        <v>2.3889739663093414</v>
+      <c r="G9" s="3">
+        <f t="shared" si="1"/>
+        <v>2.3889739663093414E-2</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>8</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="2">
         <v>5000</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="2">
         <v>5000</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="2">
         <v>5000</v>
       </c>
-      <c r="F10">
-        <f>SUM(C10:E10)</f>
+      <c r="F10" s="2">
+        <f t="shared" si="0"/>
         <v>15000</v>
       </c>
-      <c r="G10">
-        <f>(F10/$F$13)*100</f>
-        <v>9.1883614088820824</v>
+      <c r="G10" s="3">
+        <f t="shared" si="1"/>
+        <v>9.1883614088820828E-2</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>9</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="2">
         <v>6000</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="2">
         <v>6000</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="2">
         <v>6000</v>
       </c>
-      <c r="F11">
-        <f>SUM(C11:E11)</f>
+      <c r="F11" s="2">
+        <f t="shared" si="0"/>
         <v>18000</v>
       </c>
-      <c r="G11">
-        <f>(F11/$F$13)*100</f>
-        <v>11.026033690658499</v>
+      <c r="G11" s="3">
+        <f t="shared" si="1"/>
+        <v>0.11026033690658499</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>10</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="2">
         <v>450</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="2">
         <v>500</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="2">
         <v>600</v>
       </c>
-      <c r="F12">
-        <f>SUM(C12:E12)</f>
+      <c r="F12" s="2">
+        <f t="shared" si="0"/>
         <v>1550</v>
       </c>
-      <c r="G12">
-        <f>(F12/$F$13)*100</f>
-        <v>0.94946401225114863</v>
+      <c r="G12" s="3">
+        <f t="shared" si="1"/>
+        <v>9.4946401225114857E-3</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
         <v>6</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="1">
         <f>SUM(C5:C12)</f>
         <v>54550</v>
       </c>
-      <c r="D13">
-        <f t="shared" ref="D13:F13" si="0">SUM(D5:D12)</f>
+      <c r="D13" s="1">
+        <f t="shared" ref="D13:F13" si="2">SUM(D5:D12)</f>
         <v>54300</v>
       </c>
-      <c r="E13">
-        <f t="shared" si="0"/>
+      <c r="E13" s="1">
+        <f t="shared" si="2"/>
         <v>54400</v>
       </c>
-      <c r="F13">
-        <f t="shared" si="0"/>
+      <c r="F13" s="1">
+        <f t="shared" si="2"/>
         <v>163250</v>
       </c>
-      <c r="G13">
-        <f>(F13/$F$13)*100</f>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B14" t="s">
+      <c r="G13" s="3">
+        <f>(F13/$F$13)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B15" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C14">
+      <c r="C15">
         <f>MIN(C5:C12)</f>
         <v>450</v>
       </c>
-      <c r="D14">
+      <c r="D15">
         <f>MIN(D5:D12)</f>
         <v>500</v>
       </c>
-      <c r="E14">
+      <c r="E15">
         <f>MIN(E5:E12)</f>
         <v>600</v>
       </c>
-      <c r="F14">
+      <c r="F15">
         <f>MIN(F5:F12)</f>
         <v>1550</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B15" t="s">
+    <row r="16" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B16" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C15">
+      <c r="C16">
         <f>MAX(C5:C12)</f>
         <v>19000</v>
       </c>
-      <c r="D15">
+      <c r="D16">
         <f>MAX(D5:D12)</f>
         <v>19000</v>
       </c>
-      <c r="E15">
+      <c r="E16">
         <f>MAX(E5:E12)</f>
         <v>19000</v>
       </c>
-      <c r="F15">
+      <c r="F16">
         <f>MAX(F5:F12)</f>
         <v>57000</v>
       </c>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B16" t="s">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B17" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C16">
+      <c r="C17">
         <f>AVERAGE(C5:C12)</f>
         <v>6818.75</v>
       </c>
-      <c r="D16">
+      <c r="D17">
         <f>AVERAGE(D5:D12)</f>
         <v>6787.5</v>
       </c>
-      <c r="E16">
+      <c r="E17">
         <f>AVERAGE(E5:E12)</f>
         <v>6800</v>
       </c>
-      <c r="F16">
+      <c r="F17">
         <f>AVERAGE(F5:F12)</f>
         <v>20406.25</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B17" t="s">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B18" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C17">
+      <c r="C18">
         <f>COUNT(C5:C12)</f>
         <v>8</v>
       </c>
-      <c r="D17">
+      <c r="D18">
         <f>COUNT(D5:D12)</f>
         <v>8</v>
       </c>
-      <c r="E17">
+      <c r="E18">
         <f>COUNT(E5:E12)</f>
         <v>8</v>
       </c>
-      <c r="F17">
+      <c r="F18">
         <f>COUNT(F5:F12)</f>
         <v>8</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:G2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="C13:E13 C14:E17" formulaRange="1"/>
+    <ignoredError sqref="C13:E13 C15:E18" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C881B40-3868-B64D-BC40-E4666107B0E3}">
-  <dimension ref="A1:F17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1">
-        <v>45658</v>
-      </c>
-      <c r="C3" s="1">
-        <v>45689</v>
-      </c>
-      <c r="D3" s="1">
-        <v>45717</v>
-      </c>
-      <c r="E3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4">
-        <v>19000</v>
-      </c>
-      <c r="C4">
-        <v>19000</v>
-      </c>
-      <c r="D4">
-        <v>19000</v>
-      </c>
-      <c r="E4">
-        <f>SUM(B4:D4)</f>
-        <v>57000</v>
-      </c>
-      <c r="F4" t="e">
-        <f>(E4/$H$14)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5">
-        <v>600</v>
-      </c>
-      <c r="C5">
-        <v>600</v>
-      </c>
-      <c r="D5">
-        <v>600</v>
-      </c>
-      <c r="E5">
-        <f t="shared" ref="E5:E11" si="0">SUM(B5:D5)</f>
-        <v>1800</v>
-      </c>
-      <c r="F5" t="e">
-        <f>(E5/$H$14)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6">
-        <v>8000</v>
-      </c>
-      <c r="C6">
-        <v>7000</v>
-      </c>
-      <c r="D6">
-        <v>8000</v>
-      </c>
-      <c r="E6">
-        <f t="shared" si="0"/>
-        <v>23000</v>
-      </c>
-      <c r="F6" t="e">
-        <f>(E6/$H$14)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7">
-        <v>14000</v>
-      </c>
-      <c r="C7">
-        <v>15000</v>
-      </c>
-      <c r="D7">
-        <v>14000</v>
-      </c>
-      <c r="E7">
-        <f t="shared" si="0"/>
-        <v>43000</v>
-      </c>
-      <c r="F7" t="e">
-        <f>(E7/$H$14)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>1500</v>
-      </c>
-      <c r="C8">
-        <v>1200</v>
-      </c>
-      <c r="D8">
-        <v>1200</v>
-      </c>
-      <c r="E8">
-        <f t="shared" si="0"/>
-        <v>3900</v>
-      </c>
-      <c r="F8" t="e">
-        <f>(E8/$H$14)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>5000</v>
-      </c>
-      <c r="C9">
-        <v>5000</v>
-      </c>
-      <c r="D9">
-        <v>5000</v>
-      </c>
-      <c r="E9">
-        <f t="shared" si="0"/>
-        <v>15000</v>
-      </c>
-      <c r="F9" t="e">
-        <f>(E9/$H$14)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>6000</v>
-      </c>
-      <c r="C10">
-        <v>6000</v>
-      </c>
-      <c r="D10">
-        <v>6000</v>
-      </c>
-      <c r="E10">
-        <f t="shared" si="0"/>
-        <v>18000</v>
-      </c>
-      <c r="F10" t="e">
-        <f>(E10/$H$14)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>450</v>
-      </c>
-      <c r="C11">
-        <v>500</v>
-      </c>
-      <c r="D11">
-        <v>600</v>
-      </c>
-      <c r="E11">
-        <f t="shared" si="0"/>
-        <v>1550</v>
-      </c>
-      <c r="F11" t="e">
-        <f>(E11/$H$14)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12">
-        <f>SUM(B4:B11)</f>
-        <v>54550</v>
-      </c>
-      <c r="C12">
-        <f t="shared" ref="C12:E12" si="1">SUM(C4:C11)</f>
-        <v>54300</v>
-      </c>
-      <c r="D12">
-        <f t="shared" si="1"/>
-        <v>54400</v>
-      </c>
-      <c r="E12">
-        <f t="shared" si="1"/>
-        <v>163250</v>
-      </c>
-      <c r="F12" t="e">
-        <f>(E12/$H$14)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14">
-        <f>MIN(B4:B11)</f>
-        <v>450</v>
-      </c>
-      <c r="C14">
-        <f>MIN(C4:C11)</f>
-        <v>500</v>
-      </c>
-      <c r="D14">
-        <f>MIN(D4:D11)</f>
-        <v>600</v>
-      </c>
-      <c r="E14">
-        <f>MIN(E4:E11)</f>
-        <v>1550</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15">
-        <f>MAX(B4:B11)</f>
-        <v>19000</v>
-      </c>
-      <c r="C15">
-        <f>MAX(C4:C11)</f>
-        <v>19000</v>
-      </c>
-      <c r="D15">
-        <f>MAX(D4:D11)</f>
-        <v>19000</v>
-      </c>
-      <c r="E15">
-        <f>MAX(E4:E11)</f>
-        <v>57000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16">
-        <f>AVERAGE(B4:B11)</f>
-        <v>6818.75</v>
-      </c>
-      <c r="C16">
-        <f>AVERAGE(C4:C11)</f>
-        <v>6787.5</v>
-      </c>
-      <c r="D16">
-        <f>AVERAGE(D4:D11)</f>
-        <v>6800</v>
-      </c>
-      <c r="E16">
-        <f>AVERAGE(E4:E11)</f>
-        <v>20406.25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17">
-        <f>COUNT(B4:B11)</f>
-        <v>8</v>
-      </c>
-      <c r="C17">
-        <f>COUNT(C4:C11)</f>
-        <v>8</v>
-      </c>
-      <c r="D17">
-        <f>COUNT(D4:D11)</f>
-        <v>8</v>
-      </c>
-      <c r="E17">
-        <f>COUNT(E4:E11)</f>
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
formatting and moving chart to another worksheet
</commit_message>
<xml_diff>
--- a/excel/excel-101/MonthlyBudget.xlsx
+++ b/excel/excel-101/MonthlyBudget.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rajkhare/Raj/Udemy/ms-office/excel/excel-101/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{313A428E-D099-484F-817A-D324FEFA96C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF04E94-83E8-CF47-A4EC-923E6E29881E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16720" xr2:uid="{61CE2942-B3C2-844E-8245-A989A6B80F58}"/>
   </bookViews>
   <sheets>
-    <sheet name="Monthly Budget" sheetId="1" r:id="rId1"/>
+    <sheet name="Chart Monthly Budget" sheetId="3" r:id="rId1"/>
+    <sheet name="Monthly Budget" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
-  <si>
-    <t>Monthly Budget</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>Bills</t>
   </si>
@@ -83,6 +81,12 @@
   </si>
   <si>
     <t>COUNT</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>2025 Monthly Budget</t>
   </si>
 </sst>
 </file>
@@ -243,6 +247,17 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:strRef>
+          <c:f>'Monthly Budget'!$B$2:$G$2</c:f>
+          <c:strCache>
+            <c:ptCount val="6"/>
+            <c:pt idx="0">
+              <c:v>2025 Monthly Budget</c:v>
+            </c:pt>
+          </c:strCache>
+        </c:strRef>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -256,13 +271,19 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
                 </a:schemeClr>
               </a:solidFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="40000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
@@ -294,13 +315,42 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
@@ -341,7 +391,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F4B4-5E43-92F4-39D958580ABC}"/>
+              <c16:uniqueId val="{00000000-4FB0-DE45-8719-85C44EDC644F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -360,13 +410,42 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2"/>
-            </a:solidFill>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent2">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent2">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
@@ -407,7 +486,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-F4B4-5E43-92F4-39D958580ABC}"/>
+              <c16:uniqueId val="{00000001-4FB0-DE45-8719-85C44EDC644F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -426,13 +505,42 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent3"/>
-            </a:solidFill>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent3">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent3">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent3">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
@@ -473,7 +581,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000009-F4B4-5E43-92F4-39D958580ABC}"/>
+              <c16:uniqueId val="{00000002-4FB0-DE45-8719-85C44EDC644F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -492,13 +600,42 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent4"/>
-            </a:solidFill>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent4">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent4">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent4">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
@@ -539,7 +676,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000A-F4B4-5E43-92F4-39D958580ABC}"/>
+              <c16:uniqueId val="{00000003-4FB0-DE45-8719-85C44EDC644F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -558,13 +695,42 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent5"/>
-            </a:solidFill>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent5">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent5">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
@@ -605,7 +771,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-F4B4-5E43-92F4-39D958580ABC}"/>
+              <c16:uniqueId val="{00000004-4FB0-DE45-8719-85C44EDC644F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -624,13 +790,42 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent6"/>
-            </a:solidFill>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent6">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent6">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
@@ -671,7 +866,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000C-F4B4-5E43-92F4-39D958580ABC}"/>
+              <c16:uniqueId val="{00000005-4FB0-DE45-8719-85C44EDC644F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -690,15 +885,45 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1">
-                <a:lumMod val="60000"/>
-              </a:schemeClr>
-            </a:solidFill>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
@@ -739,7 +964,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000D-F4B4-5E43-92F4-39D958580ABC}"/>
+              <c16:uniqueId val="{00000006-4FB0-DE45-8719-85C44EDC644F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -758,15 +983,45 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2">
-                <a:lumMod val="60000"/>
-              </a:schemeClr>
-            </a:solidFill>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="60000"/>
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="60000"/>
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="60000"/>
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
@@ -807,7 +1062,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000E-F4B4-5E43-92F4-39D958580ABC}"/>
+              <c16:uniqueId val="{00000007-4FB0-DE45-8719-85C44EDC644F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -819,8 +1074,8 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:gapWidth val="219"/>
-        <c:overlap val="-27"/>
+        <c:gapWidth val="100"/>
+        <c:overlap val="-24"/>
         <c:axId val="74791807"/>
         <c:axId val="2047288064"/>
       </c:barChart>
@@ -832,16 +1087,16 @@
         <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:numFmt formatCode="mmm\-yyyy" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
+        <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
+              <a:schemeClr val="lt1">
+                <a:lumMod val="95000"/>
+                <a:alpha val="54000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:round/>
@@ -853,11 +1108,10 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -886,9 +1140,9 @@
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
+                  <a:alpha val="10000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:round/>
@@ -914,9 +1168,8 @@
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -940,7 +1193,7 @@
       </c:spPr>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="b"/>
+      <c:legendPos val="t"/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -954,11 +1207,10 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="85000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
@@ -982,17 +1234,28 @@
     </c:extLst>
   </c:chart>
   <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="85000"/>
+            <a:lumOff val="15000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
+    <a:ln>
+      <a:noFill/>
     </a:ln>
     <a:effectLst/>
   </c:spPr>
@@ -1006,11 +1269,6 @@
       <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
 </c:chartSpace>
 </file>
 
@@ -1055,35 +1313,33 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="209">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -1091,26 +1347,34 @@
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+  <cs:chartArea>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="85000"/>
+              <a:lumOff val="15000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
     </cs:spPr>
     <cs:defRPr sz="1000" kern="1200"/>
   </cs:chartArea>
@@ -1119,9 +1383,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -1140,14 +1403,6 @@
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
@@ -1156,35 +1411,35 @@
   </cs:dataLabelCallout>
   <cs:dataPoint>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="28575" cap="rnd">
+      <a:ln w="34925" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -1196,30 +1451,31 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
   <cs:dataPointWireframe>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -1235,21 +1491,18 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
@@ -1259,20 +1512,20 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
         </a:schemeClr>
       </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -1283,17 +1536,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
+        <a:prstDash val="dash"/>
       </a:ln>
     </cs:spPr>
   </cs:dropLine>
@@ -1302,14 +1555,13 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -1321,28 +1573,22 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
   </cs:floor>
   <cs:gridlineMajor>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="10000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -1354,17 +1600,16 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln>
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="5000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:gridlineMinor>
@@ -1373,17 +1618,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
+        <a:prstDash val="dash"/>
       </a:ln>
     </cs:spPr>
   </cs:hiLoLine>
@@ -1392,17 +1637,16 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:leaderLine>
@@ -1411,27 +1655,26 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+  <cs:plotArea>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+  <cs:plotArea3D>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:plotArea3D>
   <cs:seriesAxis>
@@ -1439,11 +1682,21 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:seriesAxis>
   <cs:seriesLine>
@@ -1451,14 +1704,14 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -1470,12 +1723,19 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="95000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:defRPr>
   </cs:title>
   <cs:trendline>
     <cs:lnRef idx="0">
@@ -1484,14 +1744,13 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="19050" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:prstDash val="sysDot"/>
       </a:ln>
     </cs:spPr>
   </cs:trendline>
@@ -1500,9 +1759,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -1512,7 +1770,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
@@ -1520,9 +1778,9 @@
       </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -1533,9 +1791,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -1545,16 +1802,18 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
   </cs:wall>
 </cs:chartStyle>
+</file>
+
+<file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{95C9785A-194E-7F4D-BAC7-855406E9F469}">
+  <sheetPr/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</chartsheet>
 </file>
 
 <file path=xl/diagrams/colors1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2662,8 +2921,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="342892" y="0"/>
-          <a:ext cx="3886112" cy="2767361"/>
+          <a:off x="342574" y="0"/>
+          <a:ext cx="3882514" cy="2767361"/>
         </a:xfrm>
         <a:prstGeom prst="rightArrow">
           <a:avLst/>
@@ -2702,8 +2961,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="4911" y="830208"/>
-          <a:ext cx="1471579" cy="1106944"/>
+          <a:off x="4906" y="830208"/>
+          <a:ext cx="1470216" cy="1106944"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -2805,8 +3064,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="58948" y="884245"/>
-        <a:ext cx="1363505" cy="998870"/>
+        <a:off x="58943" y="884245"/>
+        <a:ext cx="1362142" cy="998870"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{59C49F4E-C86E-FD4A-81A5-F3F3DE96EC27}">
@@ -2816,8 +3075,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="1550158" y="830208"/>
-          <a:ext cx="1471579" cy="1106944"/>
+          <a:off x="1548723" y="830208"/>
+          <a:ext cx="1470216" cy="1106944"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -2919,8 +3178,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="1604195" y="884245"/>
-        <a:ext cx="1363505" cy="998870"/>
+        <a:off x="1602760" y="884245"/>
+        <a:ext cx="1362142" cy="998870"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{652C8676-5948-E34F-A9C6-49D86CD1B403}">
@@ -2930,8 +3189,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="3095406" y="830208"/>
-          <a:ext cx="1471579" cy="1106944"/>
+          <a:off x="3092540" y="830208"/>
+          <a:ext cx="1470216" cy="1106944"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -2997,8 +3256,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="3149443" y="884245"/>
-        <a:ext cx="1363505" cy="998870"/>
+        <a:off x="3146577" y="884245"/>
+        <a:ext cx="1362142" cy="998870"/>
       </dsp:txXfrm>
     </dsp:sp>
   </dsp:spTree>
@@ -4195,18 +4454,51 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:absoluteAnchor>
+    <xdr:pos x="0" y="0"/>
+    <xdr:ext cx="9309919" cy="6073468"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4BA4EC7B-EB95-3634-765A-5B88E09CA215}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:absoluteAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>744247</xdr:colOff>
+      <xdr:colOff>354781</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>33757</xdr:rowOff>
+      <xdr:rowOff>25290</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>37758</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>732025</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>442622</xdr:rowOff>
+      <xdr:rowOff>434155</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4235,8 +4527,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1099301" y="231768"/>
-          <a:ext cx="372328" cy="408865"/>
+          <a:off x="710381" y="228490"/>
+          <a:ext cx="377244" cy="408865"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4415,42 +4707,6 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/diagram">
           <dgm:relIds xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:dm="rId2" r:lo="rId3" r:qs="rId4" r:cs="rId5"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>136345</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>113577</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>642796</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>32420</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C560FC6F-0728-A39F-0C19-12C28A7BF161}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4756,7 +5012,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53CFA12A-055A-DD46-B8BC-7BBA25CD28AE}">
-  <dimension ref="B1:G18"/>
+  <dimension ref="B1:K18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.6640625" customWidth="1"/>
@@ -4766,12 +5022,12 @@
     <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.2">
       <c r="F1" s="7"/>
     </row>
-    <row r="2" spans="2:7" ht="37" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="2:11" ht="37" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="8" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
@@ -4779,10 +5035,10 @@
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
     </row>
-    <row r="3" spans="2:7" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="2:7" ht="26" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:11" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="4" spans="2:11" ht="26" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" s="6">
         <v>45658</v>
@@ -4794,15 +5050,15 @@
         <v>45717</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:11" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" s="1">
         <v>19000</v>
@@ -4821,10 +5077,13 @@
         <f>(F5/$F$13)</f>
         <v>0.34915773353751917</v>
       </c>
+      <c r="K5" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C6" s="2">
         <v>600</v>
@@ -4844,9 +5103,9 @@
         <v>1.1026033690658498E-2</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C7" s="2">
         <v>8000</v>
@@ -4866,9 +5125,9 @@
         <v>0.14088820826952528</v>
       </c>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8" s="2">
         <v>14000</v>
@@ -4888,9 +5147,9 @@
         <v>0.26339969372128635</v>
       </c>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C9" s="2">
         <v>1500</v>
@@ -4910,9 +5169,9 @@
         <v>2.3889739663093414E-2</v>
       </c>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C10" s="2">
         <v>5000</v>
@@ -4932,9 +5191,9 @@
         <v>9.1883614088820828E-2</v>
       </c>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C11" s="2">
         <v>6000</v>
@@ -4954,9 +5213,9 @@
         <v>0.11026033690658499</v>
       </c>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C12" s="2">
         <v>450</v>
@@ -4976,9 +5235,9 @@
         <v>9.4946401225114857E-3</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C13" s="1">
         <f>SUM(C5:C12)</f>
@@ -5001,9 +5260,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B15" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C15">
         <f>MIN(C5:C12)</f>
@@ -5022,9 +5281,9 @@
         <v>1550</v>
       </c>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B16" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C16">
         <f>MAX(C5:C12)</f>
@@ -5045,7 +5304,7 @@
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B17" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C17">
         <f>AVERAGE(C5:C12)</f>
@@ -5066,7 +5325,7 @@
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B18" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C18">
         <f>COUNT(C5:C12)</f>

</xml_diff>